<commit_message>
Build site at 2021-05-12 15:42:42 UTC
</commit_message>
<xml_diff>
--- a/_Drive/Publicacoes/baptista.xlsx
+++ b/_Drive/Publicacoes/baptista.xlsx
@@ -4,7 +4,7 @@
   <fileVersion lastEdited="4" lowestEdited="4" rupBuild="3820"/>
   <workbookPr date1904="0"/>
   <bookViews>
-    <workbookView activeTab="0"/>
+    <workbookView activeTab="0" windowWidth="14400" windowHeight="6300"/>
   </bookViews>
   <sheets>
     <sheet name="baptista.doi" sheetId="1" r:id="rId1"/>
@@ -18,11 +18,29 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="1" count="1">
+  <si>
+    <t>DOI</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <b val="0"/>
+      <i val="0"/>
+      <u val="none"/>
+      <color rgb="FF000000"/>
+      <name val="Sans"/>
+      <vertAlign val="baseline"/>
+      <sz val="10"/>
+      <strike val="0"/>
+    </font>
+    <font>
+      <b val="1"/>
       <i val="0"/>
       <u val="none"/>
       <color rgb="FF000000"/>
@@ -62,8 +80,12 @@
       <protection locked="1" hidden="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="1" applyNumberFormat="1" fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0" textRotation="0" indent="0"/>
+      <protection locked="1" hidden="0"/>
+    </xf>
+    <xf applyAlignment="1" applyBorder="1" applyFont="1" applyFill="1" applyNumberFormat="1" fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0" textRotation="0" indent="0"/>
       <protection locked="1" hidden="0"/>
     </xf>
@@ -76,350 +98,356 @@
   <sheetPr>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A49"/>
+  <dimension ref="A1:A50"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="256" style="0" width="9.142307692307693"/>
+    <col min="1" max="1" style="0" width="39.711899038461546" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" style="0" width="9.142307692307693"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>10.1016/j.ijfatigue.2016.04.018</t>
-        </is>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="inlineStr">
         <is>
-          <t>10.1016/j.proeng.2010.03.178</t>
+          <t>10.1016/j.ijfatigue.2016.04.018</t>
         </is>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10.1016/j.engfailanal.2006.11.053</t>
+          <t>10.1016/j.proeng.2010.03.178</t>
         </is>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="inlineStr">
         <is>
-          <t>10.1007/s40430-019-1821-9</t>
+          <t>10.1016/j.engfailanal.2006.11.053</t>
         </is>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10.1016/j.prostr.2019.08.054</t>
+          <t>10.1007/s40430-019-1821-9</t>
         </is>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/amr.1135.167</t>
+          <t>10.1016/j.prostr.2019.08.054</t>
         </is>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10.17563/rbav.v34i1.939</t>
+          <t>10.4028/www.scientific.net/amr.1135.167</t>
         </is>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="inlineStr">
         <is>
-          <t>10.1243/14644207JMDA122</t>
+          <t>10.17563/rbav.v34i1.939</t>
         </is>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10.20906/CPS/COB-2015-1461</t>
+          <t>10.1243/14644207JMDA122</t>
         </is>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="inlineStr">
         <is>
-          <t>10.1016/j.proeng.2010.03.205</t>
+          <t>10.20906/CPS/COB-2015-1461</t>
         </is>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="inlineStr">
         <is>
-          <t>10.20906/CPS/COB-2015-0858</t>
+          <t>10.1016/j.proeng.2010.03.205</t>
         </is>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/msf.805.204</t>
+          <t>10.20906/CPS/COB-2015-0858</t>
         </is>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" t="inlineStr">
         <is>
-          <t>10.1590/0370-44672019740154</t>
+          <t>10.4028/www.scientific.net/msf.805.204</t>
         </is>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/KEM.713.30</t>
+          <t>10.1590/0370-44672019740154</t>
         </is>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" t="inlineStr">
         <is>
-          <t>10.1016/j.ceramint.2012.08.093</t>
+          <t>10.4028/www.scientific.net/KEM.713.30</t>
         </is>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10.1016/j.proeng.2011.04.342</t>
+          <t>10.1016/j.ceramint.2012.08.093</t>
         </is>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/AMR.891-892.615</t>
+          <t>10.1016/j.proeng.2011.04.342</t>
         </is>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="inlineStr">
         <is>
-          <t>10.1007/s40430-014-0175-6</t>
+          <t>10.4028/www.scientific.net/AMR.891-892.615</t>
         </is>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" t="inlineStr">
         <is>
-          <t>10.1016/j.ijfatigue.2004.01.011</t>
+          <t>10.1007/s40430-014-0175-6</t>
         </is>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" t="inlineStr">
         <is>
-          <t>10.1016/j.proeng.2011.04.339</t>
+          <t>10.1016/j.ijfatigue.2004.01.011</t>
         </is>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/AMR.891-892.1507</t>
+          <t>10.1016/j.proeng.2011.04.339</t>
         </is>
       </c>
     </row>
     <row r="22" spans="1:1">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/kem.754.248</t>
+          <t>10.4028/www.scientific.net/AMR.891-892.1507</t>
         </is>
       </c>
     </row>
     <row r="23" spans="1:1">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10.1016/j.proeng.2011.04.343</t>
+          <t>10.4028/www.scientific.net/kem.754.248</t>
         </is>
       </c>
     </row>
     <row r="24" spans="1:1">
       <c r="A24" t="inlineStr">
         <is>
-          <t>10.5028/jatm.v5i2.219</t>
+          <t>10.1016/j.proeng.2011.04.343</t>
         </is>
       </c>
     </row>
     <row r="25" spans="1:1">
       <c r="A25" t="inlineStr">
         <is>
-          <t>10.1016/j.jmrt.2021.01.038</t>
+          <t>10.5028/jatm.v5i2.219</t>
         </is>
       </c>
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="inlineStr">
         <is>
-          <t>10.1016/j.msea.2006.10.124</t>
+          <t>10.1016/j.jmrt.2021.01.038</t>
         </is>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/AMR.891-892.1335</t>
+          <t>10.1016/j.msea.2006.10.124</t>
         </is>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="inlineStr">
         <is>
-          <t>10.17563/rbav.v34i2.956</t>
+          <t>10.4028/www.scientific.net/AMR.891-892.1335</t>
         </is>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" t="inlineStr">
         <is>
-          <t>10.1016/j.jmrt.2013.10.005</t>
+          <t>10.17563/rbav.v34i2.956</t>
         </is>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" t="inlineStr">
         <is>
-          <t>10.3390/met9050589</t>
+          <t>10.1016/j.jmrt.2013.10.005</t>
         </is>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/MSF.727-728.945</t>
+          <t>10.3390/met9050589</t>
         </is>
       </c>
     </row>
     <row r="32" spans="1:1">
       <c r="A32" t="inlineStr">
         <is>
-          <t>10.1016/j.matdes.2008.08.010</t>
+          <t>10.4028/www.scientific.net/MSF.727-728.945</t>
         </is>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" t="inlineStr">
         <is>
-          <t>10.1051/matecconf/202032111095</t>
+          <t>10.1016/j.matdes.2008.08.010</t>
         </is>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" t="inlineStr">
         <is>
-          <t>10.1016/j.proeng.2011.04.220</t>
+          <t>10.1051/matecconf/202032111095</t>
         </is>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" t="inlineStr">
         <is>
-          <t>10.1088/2053-1591/ab6c8f</t>
+          <t>10.1016/j.proeng.2011.04.220</t>
         </is>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/MSF.636-637.47</t>
+          <t>10.1088/2053-1591/ab6c8f</t>
         </is>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/kem.754.43</t>
+          <t>10.4028/www.scientific.net/MSF.636-637.47</t>
         </is>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" t="inlineStr">
         <is>
-          <t>10.1590/0370-44672018720157</t>
+          <t>10.4028/www.scientific.net/kem.754.43</t>
         </is>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" t="inlineStr">
         <is>
-          <t>10.1016/j.proeng.2010.03.206</t>
+          <t>10.1590/0370-44672018720157</t>
         </is>
       </c>
     </row>
     <row r="40" spans="1:1">
       <c r="A40" t="inlineStr">
         <is>
-          <t>10.20906/CPS/COB-2015-0934</t>
+          <t>10.1016/j.proeng.2010.03.206</t>
         </is>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" t="inlineStr">
         <is>
-          <t>10.1016/j.mechmat.2012.04.003</t>
+          <t>10.20906/CPS/COB-2015-0934</t>
         </is>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" t="inlineStr">
         <is>
-          <t>10.1016/j.jmbbm.2014.06.011</t>
+          <t>10.1016/j.mechmat.2012.04.003</t>
         </is>
       </c>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" t="inlineStr">
         <is>
-          <t>10.1590/s0366-69132014000100006</t>
+          <t>10.1016/j.jmbbm.2014.06.011</t>
         </is>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" t="inlineStr">
         <is>
-          <t>10.1177/0021998310376098</t>
+          <t>10.1590/s0366-69132014000100006</t>
         </is>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/AMR.891-892.1785</t>
+          <t>10.1177/0021998310376098</t>
         </is>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" t="inlineStr">
         <is>
-          <t>10.1016/j.proeng.2011.04.202</t>
+          <t>10.4028/www.scientific.net/AMR.891-892.1785</t>
         </is>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" t="inlineStr">
         <is>
-          <t>10.4028/www.scientific.net/msf.869.503</t>
+          <t>10.1016/j.proeng.2011.04.202</t>
         </is>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" t="inlineStr">
         <is>
-          <t>10.1016/j.prostr.2019.08.043</t>
+          <t>10.4028/www.scientific.net/msf.869.503</t>
         </is>
       </c>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" t="inlineStr">
+        <is>
+          <t>10.1016/j.prostr.2019.08.043</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" t="inlineStr">
         <is>
           <t>10.4028/www.scientific.net/AMR.891-892.1767</t>
         </is>

</xml_diff>